<commit_message>
Narrow duplicate identity to the client's own row identity
</commit_message>
<xml_diff>
--- a/inst/fixtures/Vega/source/PCG/Vega/VP-2_Depósito_de_Relaves_Vega.xlsx
+++ b/inst/fixtures/Vega/source/PCG/Vega/VP-2_Depósito_de_Relaves_Vega.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="312">
   <si>
     <t>MONITOREO DE PIEZÓMETROS</t>
   </si>
@@ -427,247 +427,235 @@
     <t>-22.05</t>
   </si>
   <si>
-    <t>0.55903</t>
-  </si>
-  <si>
-    <t>22.02</t>
+    <t>13</t>
+  </si>
+  <si>
+    <t>45304</t>
+  </si>
+  <si>
+    <t>0.52292</t>
+  </si>
+  <si>
+    <t>0.24</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>45335</t>
+  </si>
+  <si>
+    <t>0.41875</t>
+  </si>
+  <si>
+    <t>21.72</t>
+  </si>
+  <si>
+    <t>3576.63</t>
+  </si>
+  <si>
+    <t>0.68</t>
+  </si>
+  <si>
+    <t>0.09</t>
+  </si>
+  <si>
+    <t>-21.72</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>45365</t>
+  </si>
+  <si>
+    <t>0.40069</t>
+  </si>
+  <si>
+    <t>21.38</t>
+  </si>
+  <si>
+    <t>3576.97</t>
+  </si>
+  <si>
+    <t>1.02</t>
+  </si>
+  <si>
+    <t>0.34</t>
+  </si>
+  <si>
+    <t>-21.38</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>45393</t>
+  </si>
+  <si>
+    <t>0.41528</t>
+  </si>
+  <si>
+    <t>21.05</t>
+  </si>
+  <si>
+    <t>3577.30</t>
+  </si>
+  <si>
+    <t>1.35</t>
+  </si>
+  <si>
+    <t>0.33</t>
+  </si>
+  <si>
+    <t>-21.05</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>45431</t>
+  </si>
+  <si>
+    <t>0.45764</t>
+  </si>
+  <si>
+    <t>0.18</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>45459</t>
+  </si>
+  <si>
+    <t>0.38889</t>
+  </si>
+  <si>
+    <t>20.98</t>
+  </si>
+  <si>
+    <t>3577.37</t>
+  </si>
+  <si>
+    <t>1.42</t>
+  </si>
+  <si>
+    <t>-0.11</t>
+  </si>
+  <si>
+    <t>-20.98</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>45490</t>
+  </si>
+  <si>
+    <t>0.41389</t>
+  </si>
+  <si>
+    <t>24.40</t>
+  </si>
+  <si>
+    <t>22.85</t>
+  </si>
+  <si>
+    <t>3600.35</t>
+  </si>
+  <si>
+    <t>3577.50</t>
+  </si>
+  <si>
+    <t>1.55</t>
+  </si>
+  <si>
+    <t>0.13</t>
+  </si>
+  <si>
+    <t>-22.85</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>45516</t>
+  </si>
+  <si>
+    <t>0.38681</t>
+  </si>
+  <si>
+    <t>23.10</t>
+  </si>
+  <si>
+    <t>3577.25</t>
+  </si>
+  <si>
+    <t>1.30</t>
+  </si>
+  <si>
+    <t>-23.10</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>45553</t>
+  </si>
+  <si>
+    <t>0.48125</t>
+  </si>
+  <si>
+    <t>23.47</t>
+  </si>
+  <si>
+    <t>-0.37</t>
+  </si>
+  <si>
+    <t>-23.47</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>45584</t>
+  </si>
+  <si>
+    <t>0.50764</t>
+  </si>
+  <si>
+    <t>23.78</t>
+  </si>
+  <si>
+    <t>3576.57</t>
+  </si>
+  <si>
+    <t>0.62</t>
+  </si>
+  <si>
+    <t>-0.31</t>
+  </si>
+  <si>
+    <t>-23.78</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>45615</t>
+  </si>
+  <si>
+    <t>0.35903</t>
+  </si>
+  <si>
+    <t>24.02</t>
   </si>
   <si>
     <t>3576.33</t>
   </si>
   <si>
     <t>0.38</t>
-  </si>
-  <si>
-    <t>0.03</t>
-  </si>
-  <si>
-    <t>-22.02</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>45304</t>
-  </si>
-  <si>
-    <t>0.52292</t>
-  </si>
-  <si>
-    <t>0.24</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>45335</t>
-  </si>
-  <si>
-    <t>0.41875</t>
-  </si>
-  <si>
-    <t>21.72</t>
-  </si>
-  <si>
-    <t>3576.63</t>
-  </si>
-  <si>
-    <t>0.68</t>
-  </si>
-  <si>
-    <t>0.09</t>
-  </si>
-  <si>
-    <t>-21.72</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>45365</t>
-  </si>
-  <si>
-    <t>0.40069</t>
-  </si>
-  <si>
-    <t>21.38</t>
-  </si>
-  <si>
-    <t>3576.97</t>
-  </si>
-  <si>
-    <t>1.02</t>
-  </si>
-  <si>
-    <t>0.34</t>
-  </si>
-  <si>
-    <t>-21.38</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>45393</t>
-  </si>
-  <si>
-    <t>0.41528</t>
-  </si>
-  <si>
-    <t>21.05</t>
-  </si>
-  <si>
-    <t>3577.30</t>
-  </si>
-  <si>
-    <t>1.35</t>
-  </si>
-  <si>
-    <t>0.33</t>
-  </si>
-  <si>
-    <t>-21.05</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>45431</t>
-  </si>
-  <si>
-    <t>0.45764</t>
-  </si>
-  <si>
-    <t>0.18</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>45459</t>
-  </si>
-  <si>
-    <t>0.38889</t>
-  </si>
-  <si>
-    <t>20.98</t>
-  </si>
-  <si>
-    <t>3577.37</t>
-  </si>
-  <si>
-    <t>1.42</t>
-  </si>
-  <si>
-    <t>-0.11</t>
-  </si>
-  <si>
-    <t>-20.98</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>45490</t>
-  </si>
-  <si>
-    <t>0.41389</t>
-  </si>
-  <si>
-    <t>24.40</t>
-  </si>
-  <si>
-    <t>22.85</t>
-  </si>
-  <si>
-    <t>3600.35</t>
-  </si>
-  <si>
-    <t>3577.50</t>
-  </si>
-  <si>
-    <t>1.55</t>
-  </si>
-  <si>
-    <t>0.13</t>
-  </si>
-  <si>
-    <t>-22.85</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>45516</t>
-  </si>
-  <si>
-    <t>0.38681</t>
-  </si>
-  <si>
-    <t>23.10</t>
-  </si>
-  <si>
-    <t>3577.25</t>
-  </si>
-  <si>
-    <t>1.30</t>
-  </si>
-  <si>
-    <t>-23.10</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>45553</t>
-  </si>
-  <si>
-    <t>0.48125</t>
-  </si>
-  <si>
-    <t>23.47</t>
-  </si>
-  <si>
-    <t>-0.37</t>
-  </si>
-  <si>
-    <t>-23.47</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>45584</t>
-  </si>
-  <si>
-    <t>0.50764</t>
-  </si>
-  <si>
-    <t>23.78</t>
-  </si>
-  <si>
-    <t>3576.57</t>
-  </si>
-  <si>
-    <t>0.62</t>
-  </si>
-  <si>
-    <t>-0.31</t>
-  </si>
-  <si>
-    <t>-23.78</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>45615</t>
-  </si>
-  <si>
-    <t>0.35903</t>
-  </si>
-  <si>
-    <t>24.02</t>
   </si>
   <si>
     <t>-0.24</t>
@@ -1887,13 +1875,13 @@
         <v>131</v>
       </c>
       <c r="C23" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D23" t="s">
         <v>41</v>
       </c>
       <c r="E23" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F23" t="s">
         <v>43</v>
@@ -1902,30 +1890,30 @@
         <v>44</v>
       </c>
       <c r="H23" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="I23" t="s">
-        <v>140</v>
+        <v>72</v>
       </c>
       <c r="J23" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="K23" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="N23" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:14">
       <c r="A24" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B24" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C24" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
         <v>41</v>
@@ -1946,7 +1934,7 @@
         <v>119</v>
       </c>
       <c r="J24" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="K24" t="s">
         <v>56</v>
@@ -1957,19 +1945,19 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B25" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="D25" t="s">
         <v>41</v>
       </c>
       <c r="E25" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="F25" t="s">
         <v>43</v>
@@ -1978,36 +1966,36 @@
         <v>44</v>
       </c>
       <c r="H25" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="I25" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J25" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="K25" t="s">
         <v>56</v>
       </c>
       <c r="N25" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C26" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D26" t="s">
         <v>41</v>
       </c>
       <c r="E26" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="F26" t="s">
         <v>43</v>
@@ -2016,36 +2004,36 @@
         <v>44</v>
       </c>
       <c r="H26" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="I26" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="J26" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="K26" t="s">
         <v>56</v>
       </c>
       <c r="N26" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:14">
       <c r="A27" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B27" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C27" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D27" t="s">
         <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F27" t="s">
         <v>43</v>
@@ -2054,30 +2042,30 @@
         <v>44</v>
       </c>
       <c r="H27" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="I27" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="J27" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="K27" t="s">
         <v>56</v>
       </c>
       <c r="N27" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:14">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B28" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C28" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D28" t="s">
         <v>41</v>
@@ -2098,7 +2086,7 @@
         <v>79</v>
       </c>
       <c r="J28" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="K28" t="s">
         <v>56</v>
@@ -2109,19 +2097,19 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C29" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D29" t="s">
         <v>41</v>
       </c>
       <c r="E29" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F29" t="s">
         <v>43</v>
@@ -2130,86 +2118,86 @@
         <v>44</v>
       </c>
       <c r="H29" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="I29" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="J29" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="K29" t="s">
         <v>96</v>
       </c>
       <c r="N29" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:14">
       <c r="A30" t="s">
+        <v>177</v>
+      </c>
+      <c r="B30" t="s">
+        <v>178</v>
+      </c>
+      <c r="C30" t="s">
+        <v>179</v>
+      </c>
+      <c r="D30" t="s">
+        <v>180</v>
+      </c>
+      <c r="E30" t="s">
+        <v>181</v>
+      </c>
+      <c r="F30" t="s">
+        <v>182</v>
+      </c>
+      <c r="G30" t="s">
+        <v>44</v>
+      </c>
+      <c r="H30" t="s">
         <v>183</v>
       </c>
-      <c r="B30" t="s">
+      <c r="I30" t="s">
         <v>184</v>
       </c>
-      <c r="C30" t="s">
+      <c r="J30" t="s">
         <v>185</v>
-      </c>
-      <c r="D30" t="s">
-        <v>186</v>
-      </c>
-      <c r="E30" t="s">
-        <v>187</v>
-      </c>
-      <c r="F30" t="s">
-        <v>188</v>
-      </c>
-      <c r="G30" t="s">
-        <v>44</v>
-      </c>
-      <c r="H30" t="s">
-        <v>189</v>
-      </c>
-      <c r="I30" t="s">
-        <v>190</v>
-      </c>
-      <c r="J30" t="s">
-        <v>191</v>
       </c>
       <c r="K30" t="s">
         <v>56</v>
       </c>
       <c r="N30" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="31" spans="1:14">
       <c r="A31" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B31" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C31" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D31" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E31" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="F31" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G31" t="s">
         <v>44</v>
       </c>
       <c r="H31" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="I31" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="J31" t="s">
         <v>112</v>
@@ -2218,27 +2206,27 @@
         <v>96</v>
       </c>
       <c r="N31" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="32" spans="1:14">
       <c r="A32" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B32" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C32" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="D32" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E32" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F32" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G32" t="s">
         <v>44</v>
@@ -2250,156 +2238,156 @@
         <v>63</v>
       </c>
       <c r="J32" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="K32" t="s">
         <v>96</v>
       </c>
       <c r="N32" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:14">
       <c r="A33" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" t="s">
+        <v>201</v>
+      </c>
+      <c r="C33" t="s">
+        <v>202</v>
+      </c>
+      <c r="D33" t="s">
+        <v>180</v>
+      </c>
+      <c r="E33" t="s">
+        <v>203</v>
+      </c>
+      <c r="F33" t="s">
+        <v>182</v>
+      </c>
+      <c r="G33" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" t="s">
+        <v>204</v>
+      </c>
+      <c r="I33" t="s">
+        <v>205</v>
+      </c>
+      <c r="J33" t="s">
         <v>206</v>
-      </c>
-      <c r="B33" t="s">
-        <v>207</v>
-      </c>
-      <c r="C33" t="s">
-        <v>208</v>
-      </c>
-      <c r="D33" t="s">
-        <v>186</v>
-      </c>
-      <c r="E33" t="s">
-        <v>209</v>
-      </c>
-      <c r="F33" t="s">
-        <v>188</v>
-      </c>
-      <c r="G33" t="s">
-        <v>44</v>
-      </c>
-      <c r="H33" t="s">
-        <v>210</v>
-      </c>
-      <c r="I33" t="s">
-        <v>211</v>
-      </c>
-      <c r="J33" t="s">
-        <v>212</v>
       </c>
       <c r="K33" t="s">
         <v>96</v>
       </c>
       <c r="N33" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="34" spans="1:14">
       <c r="A34" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" t="s">
+        <v>209</v>
+      </c>
+      <c r="C34" t="s">
+        <v>210</v>
+      </c>
+      <c r="D34" t="s">
+        <v>180</v>
+      </c>
+      <c r="E34" t="s">
+        <v>211</v>
+      </c>
+      <c r="F34" t="s">
+        <v>182</v>
+      </c>
+      <c r="G34" t="s">
+        <v>44</v>
+      </c>
+      <c r="H34" t="s">
+        <v>212</v>
+      </c>
+      <c r="I34" t="s">
+        <v>213</v>
+      </c>
+      <c r="J34" t="s">
         <v>214</v>
-      </c>
-      <c r="B34" t="s">
-        <v>215</v>
-      </c>
-      <c r="C34" t="s">
-        <v>216</v>
-      </c>
-      <c r="D34" t="s">
-        <v>186</v>
-      </c>
-      <c r="E34" t="s">
-        <v>217</v>
-      </c>
-      <c r="F34" t="s">
-        <v>188</v>
-      </c>
-      <c r="G34" t="s">
-        <v>44</v>
-      </c>
-      <c r="H34" t="s">
-        <v>139</v>
-      </c>
-      <c r="I34" t="s">
-        <v>140</v>
-      </c>
-      <c r="J34" t="s">
-        <v>218</v>
       </c>
       <c r="K34" t="s">
         <v>96</v>
       </c>
       <c r="N34" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="35" spans="1:14">
       <c r="A35" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" t="s">
+        <v>217</v>
+      </c>
+      <c r="C35" t="s">
+        <v>218</v>
+      </c>
+      <c r="D35" t="s">
+        <v>180</v>
+      </c>
+      <c r="E35" t="s">
+        <v>219</v>
+      </c>
+      <c r="F35" t="s">
+        <v>182</v>
+      </c>
+      <c r="G35" t="s">
+        <v>44</v>
+      </c>
+      <c r="H35" t="s">
         <v>220</v>
       </c>
-      <c r="B35" t="s">
+      <c r="I35" t="s">
         <v>221</v>
       </c>
-      <c r="C35" t="s">
-        <v>222</v>
-      </c>
-      <c r="D35" t="s">
-        <v>186</v>
-      </c>
-      <c r="E35" t="s">
-        <v>223</v>
-      </c>
-      <c r="F35" t="s">
-        <v>188</v>
-      </c>
-      <c r="G35" t="s">
-        <v>44</v>
-      </c>
-      <c r="H35" t="s">
-        <v>224</v>
-      </c>
-      <c r="I35" t="s">
-        <v>225</v>
-      </c>
       <c r="J35" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="K35" t="s">
         <v>56</v>
       </c>
       <c r="N35" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" spans="1:14">
       <c r="A36" t="s">
+        <v>223</v>
+      </c>
+      <c r="B36" t="s">
+        <v>224</v>
+      </c>
+      <c r="C36" t="s">
+        <v>225</v>
+      </c>
+      <c r="D36" t="s">
+        <v>180</v>
+      </c>
+      <c r="E36" t="s">
+        <v>226</v>
+      </c>
+      <c r="F36" t="s">
+        <v>182</v>
+      </c>
+      <c r="G36" t="s">
+        <v>44</v>
+      </c>
+      <c r="H36" t="s">
         <v>227</v>
       </c>
-      <c r="B36" t="s">
+      <c r="I36" t="s">
         <v>228</v>
-      </c>
-      <c r="C36" t="s">
-        <v>229</v>
-      </c>
-      <c r="D36" t="s">
-        <v>186</v>
-      </c>
-      <c r="E36" t="s">
-        <v>230</v>
-      </c>
-      <c r="F36" t="s">
-        <v>188</v>
-      </c>
-      <c r="G36" t="s">
-        <v>44</v>
-      </c>
-      <c r="H36" t="s">
-        <v>231</v>
-      </c>
-      <c r="I36" t="s">
-        <v>232</v>
       </c>
       <c r="J36" t="s">
         <v>87</v>
@@ -2408,103 +2396,103 @@
         <v>56</v>
       </c>
       <c r="N36" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" t="s">
+        <v>230</v>
+      </c>
+      <c r="B37" t="s">
+        <v>231</v>
+      </c>
+      <c r="C37" t="s">
+        <v>232</v>
+      </c>
+      <c r="D37" t="s">
+        <v>180</v>
+      </c>
+      <c r="E37" t="s">
+        <v>233</v>
+      </c>
+      <c r="F37" t="s">
+        <v>182</v>
+      </c>
+      <c r="G37" t="s">
+        <v>44</v>
+      </c>
+      <c r="H37" t="s">
         <v>234</v>
       </c>
-      <c r="B37" t="s">
+      <c r="I37" t="s">
         <v>235</v>
       </c>
-      <c r="C37" t="s">
+      <c r="J37" t="s">
         <v>236</v>
-      </c>
-      <c r="D37" t="s">
-        <v>186</v>
-      </c>
-      <c r="E37" t="s">
-        <v>237</v>
-      </c>
-      <c r="F37" t="s">
-        <v>188</v>
-      </c>
-      <c r="G37" t="s">
-        <v>44</v>
-      </c>
-      <c r="H37" t="s">
-        <v>238</v>
-      </c>
-      <c r="I37" t="s">
-        <v>239</v>
-      </c>
-      <c r="J37" t="s">
-        <v>240</v>
       </c>
       <c r="K37" t="s">
         <v>56</v>
       </c>
       <c r="N37" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" t="s">
+        <v>238</v>
+      </c>
+      <c r="B38" t="s">
+        <v>239</v>
+      </c>
+      <c r="C38" t="s">
+        <v>240</v>
+      </c>
+      <c r="D38" t="s">
+        <v>180</v>
+      </c>
+      <c r="E38" t="s">
+        <v>241</v>
+      </c>
+      <c r="F38" t="s">
+        <v>182</v>
+      </c>
+      <c r="G38" t="s">
+        <v>44</v>
+      </c>
+      <c r="H38" t="s">
         <v>242</v>
       </c>
-      <c r="B38" t="s">
+      <c r="I38" t="s">
         <v>243</v>
       </c>
-      <c r="C38" t="s">
+      <c r="J38" t="s">
         <v>244</v>
-      </c>
-      <c r="D38" t="s">
-        <v>186</v>
-      </c>
-      <c r="E38" t="s">
-        <v>245</v>
-      </c>
-      <c r="F38" t="s">
-        <v>188</v>
-      </c>
-      <c r="G38" t="s">
-        <v>44</v>
-      </c>
-      <c r="H38" t="s">
-        <v>246</v>
-      </c>
-      <c r="I38" t="s">
-        <v>247</v>
-      </c>
-      <c r="J38" t="s">
-        <v>248</v>
       </c>
       <c r="K38" t="s">
         <v>56</v>
       </c>
       <c r="N38" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="39" spans="1:14">
       <c r="A39" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B39" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="C39" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D39" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E39" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="F39" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G39" t="s">
         <v>44</v>
@@ -2516,270 +2504,270 @@
         <v>71</v>
       </c>
       <c r="J39" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="K39" t="s">
         <v>56</v>
       </c>
       <c r="N39" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="40" spans="1:14">
       <c r="A40" t="s">
+        <v>252</v>
+      </c>
+      <c r="B40" t="s">
+        <v>253</v>
+      </c>
+      <c r="C40" t="s">
+        <v>254</v>
+      </c>
+      <c r="D40" t="s">
+        <v>180</v>
+      </c>
+      <c r="E40" t="s">
+        <v>255</v>
+      </c>
+      <c r="F40" t="s">
+        <v>182</v>
+      </c>
+      <c r="G40" t="s">
+        <v>44</v>
+      </c>
+      <c r="H40" t="s">
         <v>256</v>
       </c>
-      <c r="B40" t="s">
+      <c r="I40" t="s">
         <v>257</v>
       </c>
-      <c r="C40" t="s">
-        <v>258</v>
-      </c>
-      <c r="D40" t="s">
-        <v>186</v>
-      </c>
-      <c r="E40" t="s">
-        <v>259</v>
-      </c>
-      <c r="F40" t="s">
-        <v>188</v>
-      </c>
-      <c r="G40" t="s">
-        <v>44</v>
-      </c>
-      <c r="H40" t="s">
-        <v>260</v>
-      </c>
-      <c r="I40" t="s">
-        <v>261</v>
-      </c>
       <c r="J40" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="K40" t="s">
         <v>56</v>
       </c>
       <c r="N40" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:14">
       <c r="A41" t="s">
+        <v>259</v>
+      </c>
+      <c r="B41" t="s">
+        <v>260</v>
+      </c>
+      <c r="C41" t="s">
+        <v>261</v>
+      </c>
+      <c r="D41" t="s">
+        <v>180</v>
+      </c>
+      <c r="E41" t="s">
+        <v>262</v>
+      </c>
+      <c r="F41" t="s">
+        <v>182</v>
+      </c>
+      <c r="G41" t="s">
+        <v>44</v>
+      </c>
+      <c r="H41" t="s">
         <v>263</v>
       </c>
-      <c r="B41" t="s">
+      <c r="I41" t="s">
         <v>264</v>
       </c>
-      <c r="C41" t="s">
+      <c r="J41" t="s">
         <v>265</v>
-      </c>
-      <c r="D41" t="s">
-        <v>186</v>
-      </c>
-      <c r="E41" t="s">
-        <v>266</v>
-      </c>
-      <c r="F41" t="s">
-        <v>188</v>
-      </c>
-      <c r="G41" t="s">
-        <v>44</v>
-      </c>
-      <c r="H41" t="s">
-        <v>267</v>
-      </c>
-      <c r="I41" t="s">
-        <v>268</v>
-      </c>
-      <c r="J41" t="s">
-        <v>269</v>
       </c>
       <c r="K41" t="s">
         <v>56</v>
       </c>
       <c r="N41" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
     </row>
     <row r="42" spans="1:14">
       <c r="A42" t="s">
+        <v>267</v>
+      </c>
+      <c r="B42" t="s">
+        <v>268</v>
+      </c>
+      <c r="C42" t="s">
+        <v>269</v>
+      </c>
+      <c r="D42" t="s">
+        <v>180</v>
+      </c>
+      <c r="E42" t="s">
+        <v>270</v>
+      </c>
+      <c r="F42" t="s">
+        <v>182</v>
+      </c>
+      <c r="G42" t="s">
+        <v>44</v>
+      </c>
+      <c r="H42" t="s">
         <v>271</v>
       </c>
-      <c r="B42" t="s">
+      <c r="I42" t="s">
         <v>272</v>
       </c>
-      <c r="C42" t="s">
+      <c r="J42" t="s">
         <v>273</v>
-      </c>
-      <c r="D42" t="s">
-        <v>186</v>
-      </c>
-      <c r="E42" t="s">
-        <v>274</v>
-      </c>
-      <c r="F42" t="s">
-        <v>188</v>
-      </c>
-      <c r="G42" t="s">
-        <v>44</v>
-      </c>
-      <c r="H42" t="s">
-        <v>275</v>
-      </c>
-      <c r="I42" t="s">
-        <v>276</v>
-      </c>
-      <c r="J42" t="s">
-        <v>277</v>
       </c>
       <c r="K42" t="s">
         <v>96</v>
       </c>
       <c r="N42" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" t="s">
+        <v>275</v>
+      </c>
+      <c r="B43" t="s">
+        <v>276</v>
+      </c>
+      <c r="C43" t="s">
+        <v>277</v>
+      </c>
+      <c r="D43" t="s">
+        <v>180</v>
+      </c>
+      <c r="E43" t="s">
+        <v>278</v>
+      </c>
+      <c r="F43" t="s">
+        <v>182</v>
+      </c>
+      <c r="G43" t="s">
+        <v>44</v>
+      </c>
+      <c r="H43" t="s">
         <v>279</v>
       </c>
-      <c r="B43" t="s">
+      <c r="I43" t="s">
         <v>280</v>
       </c>
-      <c r="C43" t="s">
+      <c r="J43" t="s">
         <v>281</v>
-      </c>
-      <c r="D43" t="s">
-        <v>186</v>
-      </c>
-      <c r="E43" t="s">
-        <v>282</v>
-      </c>
-      <c r="F43" t="s">
-        <v>188</v>
-      </c>
-      <c r="G43" t="s">
-        <v>44</v>
-      </c>
-      <c r="H43" t="s">
-        <v>283</v>
-      </c>
-      <c r="I43" t="s">
-        <v>284</v>
-      </c>
-      <c r="J43" t="s">
-        <v>285</v>
       </c>
       <c r="K43" t="s">
         <v>96</v>
       </c>
       <c r="N43" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
     </row>
     <row r="44" spans="1:14">
       <c r="A44" t="s">
+        <v>283</v>
+      </c>
+      <c r="B44" t="s">
+        <v>284</v>
+      </c>
+      <c r="C44" t="s">
+        <v>285</v>
+      </c>
+      <c r="D44" t="s">
+        <v>180</v>
+      </c>
+      <c r="E44" t="s">
+        <v>286</v>
+      </c>
+      <c r="F44" t="s">
+        <v>182</v>
+      </c>
+      <c r="G44" t="s">
+        <v>44</v>
+      </c>
+      <c r="H44" t="s">
+        <v>153</v>
+      </c>
+      <c r="I44" t="s">
+        <v>154</v>
+      </c>
+      <c r="J44" t="s">
         <v>287</v>
-      </c>
-      <c r="B44" t="s">
-        <v>288</v>
-      </c>
-      <c r="C44" t="s">
-        <v>289</v>
-      </c>
-      <c r="D44" t="s">
-        <v>186</v>
-      </c>
-      <c r="E44" t="s">
-        <v>290</v>
-      </c>
-      <c r="F44" t="s">
-        <v>188</v>
-      </c>
-      <c r="G44" t="s">
-        <v>44</v>
-      </c>
-      <c r="H44" t="s">
-        <v>159</v>
-      </c>
-      <c r="I44" t="s">
-        <v>160</v>
-      </c>
-      <c r="J44" t="s">
-        <v>291</v>
       </c>
       <c r="K44" t="s">
         <v>96</v>
       </c>
       <c r="N44" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="1:14">
       <c r="A45" t="s">
+        <v>289</v>
+      </c>
+      <c r="B45" t="s">
+        <v>290</v>
+      </c>
+      <c r="C45" t="s">
+        <v>291</v>
+      </c>
+      <c r="D45" t="s">
+        <v>180</v>
+      </c>
+      <c r="E45" t="s">
+        <v>292</v>
+      </c>
+      <c r="F45" t="s">
+        <v>182</v>
+      </c>
+      <c r="G45" t="s">
+        <v>44</v>
+      </c>
+      <c r="H45" t="s">
         <v>293</v>
       </c>
-      <c r="B45" t="s">
+      <c r="I45" t="s">
         <v>294</v>
       </c>
-      <c r="C45" t="s">
+      <c r="J45" t="s">
         <v>295</v>
-      </c>
-      <c r="D45" t="s">
-        <v>186</v>
-      </c>
-      <c r="E45" t="s">
-        <v>296</v>
-      </c>
-      <c r="F45" t="s">
-        <v>188</v>
-      </c>
-      <c r="G45" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45" t="s">
-        <v>297</v>
-      </c>
-      <c r="I45" t="s">
-        <v>298</v>
-      </c>
-      <c r="J45" t="s">
-        <v>299</v>
       </c>
       <c r="K45" t="s">
         <v>96</v>
       </c>
       <c r="N45" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="46" spans="1:14">
       <c r="A46" t="s">
+        <v>297</v>
+      </c>
+      <c r="B46" t="s">
+        <v>298</v>
+      </c>
+      <c r="C46" t="s">
+        <v>299</v>
+      </c>
+      <c r="D46" t="s">
+        <v>180</v>
+      </c>
+      <c r="E46" t="s">
+        <v>300</v>
+      </c>
+      <c r="F46" t="s">
+        <v>182</v>
+      </c>
+      <c r="G46" t="s">
+        <v>44</v>
+      </c>
+      <c r="H46" t="s">
         <v>301</v>
       </c>
-      <c r="B46" t="s">
+      <c r="I46" t="s">
         <v>302</v>
-      </c>
-      <c r="C46" t="s">
-        <v>303</v>
-      </c>
-      <c r="D46" t="s">
-        <v>186</v>
-      </c>
-      <c r="E46" t="s">
-        <v>304</v>
-      </c>
-      <c r="F46" t="s">
-        <v>188</v>
-      </c>
-      <c r="G46" t="s">
-        <v>44</v>
-      </c>
-      <c r="H46" t="s">
-        <v>305</v>
-      </c>
-      <c r="I46" t="s">
-        <v>306</v>
       </c>
       <c r="J46" t="s">
         <v>112</v>
@@ -2788,45 +2776,45 @@
         <v>96</v>
       </c>
       <c r="N46" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47" t="s">
+        <v>304</v>
+      </c>
+      <c r="B47" t="s">
+        <v>305</v>
+      </c>
+      <c r="C47" t="s">
+        <v>306</v>
+      </c>
+      <c r="D47" t="s">
+        <v>180</v>
+      </c>
+      <c r="E47" t="s">
+        <v>307</v>
+      </c>
+      <c r="F47" t="s">
+        <v>182</v>
+      </c>
+      <c r="G47" t="s">
+        <v>44</v>
+      </c>
+      <c r="H47" t="s">
         <v>308</v>
       </c>
-      <c r="B47" t="s">
+      <c r="I47" t="s">
         <v>309</v>
       </c>
-      <c r="C47" t="s">
+      <c r="J47" t="s">
         <v>310</v>
-      </c>
-      <c r="D47" t="s">
-        <v>186</v>
-      </c>
-      <c r="E47" t="s">
-        <v>311</v>
-      </c>
-      <c r="F47" t="s">
-        <v>188</v>
-      </c>
-      <c r="G47" t="s">
-        <v>44</v>
-      </c>
-      <c r="H47" t="s">
-        <v>312</v>
-      </c>
-      <c r="I47" t="s">
-        <v>313</v>
-      </c>
-      <c r="J47" t="s">
-        <v>314</v>
       </c>
       <c r="K47" t="s">
         <v>56</v>
       </c>
       <c r="N47" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>